<commit_message>
sync dashboard data for 0911 template
</commit_message>
<xml_diff>
--- a/周维度经营看板上传模板.xlsx
+++ b/周维度经营看板上传模板.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JunJun\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cwf\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="11074"/>
+    <workbookView windowWidth="21600" windowHeight="9105" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="订单数据" sheetId="1" r:id="rId1"/>
@@ -69,11 +69,21 @@
         <r>
           <rPr>
             <sz val="10"/>
+            <color rgb="FF000000"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
   - 蔡伟凤</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="宋体"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+  - 蒋一珺</t>
         </r>
       </text>
     </comment>
@@ -82,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="95">
   <si>
     <t>周次</t>
   </si>
@@ -120,6 +130,21 @@
     <t>08-06</t>
   </si>
   <si>
+    <t>08-13</t>
+  </si>
+  <si>
+    <t>08-20</t>
+  </si>
+  <si>
+    <t>08-27</t>
+  </si>
+  <si>
+    <t>09-03</t>
+  </si>
+  <si>
+    <t>09-10</t>
+  </si>
+  <si>
     <t>采购合同个数</t>
   </si>
   <si>
@@ -168,10 +193,7 @@
     <t>备注说明</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>阈值调整</t>
+    <t>明星产品清单更新</t>
   </si>
   <si>
     <t>单笔议价金额（元）</t>
@@ -238,6 +260,9 @@
   </si>
   <si>
     <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
   </si>
   <si>
     <t>模块</t>
@@ -270,6 +295,42 @@
 时间待定：自动收票——待收票（成品）</t>
   </si>
   <si>
+    <t>AI/流程优化</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI
+1、知识库:已开放给销售,16项问题待优化
+2、探索报价:任务分流内测已完成,待服务器购买后上线.
+3、待决策:所有龙虾统一API密钥，以及服务器部署
+流程优化:
+1、供应商预付款:系统增加责任人和跟踪记录,余额原因便于后续跟进,已同步试剂
+2、成品采购时可按库地或销售订单一键拆单提高采购效率。
+3、增加隔离库(如正在生产转换过程中的,以及待上架的商品个数,增加直发但未到货个数的字段,方便做应备货数量的判断
+4、增加近30天入库的个数便于后续AI对账
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI
+1、下订单：测试优化中
+2、知识库：前台详情页内容提取方案和IT沟通中
+流程优化
+1、公司自用商品采购流程优化，取消易快报
+2、提需求：①纯源开通采购单中心DEEPFLOW的查看权限；②低温商品系统需同步给仓储；③开放给销售订单中心是直发还是发仓库的查看权限；④库存信息管理增加厂家批号搜索项，便于采购查找。⑤打印单取消6个订单号的限制，根据内容调整大小；
+</t>
+  </si>
+  <si>
+    <t>08-21</t>
+  </si>
+  <si>
+    <t>①询货期和价格审批逻辑初步完成，待下周再最终确认。②、询报价录入逻辑梳理完成，待接口。③采购相关用workbuddy工具接近完成。</t>
+  </si>
+  <si>
+    <t>①workbuddy看板细节优化：预警、富余库存判定、看板升级、分仓采购与调拨逻辑区分（重要）、断货原因追溯、链接两个重要变动提醒。②龙虾报货期逻辑已确认，新增大客户下单接口需求，服务器已部署</t>
+  </si>
+  <si>
+    <t>①退换单中心：增加给仓库的备注，检查货物要求②询货期龙虾上线,详情页接口本周六做好,计量跟进的workbuddy框架搭建完成,数据采集虾上线</t>
+  </si>
+  <si>
     <t>仓库/品类</t>
   </si>
   <si>
@@ -303,6 +364,18 @@
     <t>周转天数变化(天）</t>
   </si>
   <si>
+    <t>8月库存金额</t>
+  </si>
+  <si>
+    <t>8月年营业成本</t>
+  </si>
+  <si>
+    <t>8月周转次数</t>
+  </si>
+  <si>
+    <t>8月平均周转天数</t>
+  </si>
+  <si>
     <t>主仓有阈值的明星产品</t>
   </si>
   <si>
@@ -327,28 +400,23 @@
     <t>本周小结</t>
   </si>
   <si>
-    <t>KEY-SKY断货率进一步降低到2%，新下单金额上涨81%，7月廊坊仓面积从1300平降低到1100平</t>
-  </si>
-  <si>
-    <t>08-01</t>
-  </si>
-  <si>
-    <t>08-10</t>
+    <t>①本周耗材订单环比上涨16%②仓储空间紧张,待下周转移部分商品到新飞路③明星产品重新确认,筛选原则为年度销售额超1万或毛利超2000元④计划上架MRO畅销品,已采集震坤行畅销数据,待进一步分析.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.00_ "/>
-    <numFmt numFmtId="177" formatCode="0.0%"/>
+    <numFmt numFmtId="176" formatCode="#\.0,&quot;万&quot;"/>
+    <numFmt numFmtId="177" formatCode="0_ "/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -363,9 +431,21 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="等线"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF284D79"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF08090C"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -528,6 +608,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF000000"/>
@@ -555,19 +641,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEAF3FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB2A2C7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE5B9B7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3FC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB2A2C7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -896,28 +982,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -926,185 +1003,224 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1113,41 +1229,29 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="178" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment/>
-      <extLst>
-        <ext xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" uri="{F19249F5-4A6E-446B-B59F-E2C9F2DAA1D5}">
-          <etc:displayText val="2"/>
-        </ext>
-      </extLst>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" quotePrefix="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1"/>
     <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1469,62 +1573,64 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="2"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="7"/>
   <cols>
-    <col min="6" max="6" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.3333333333333" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.1627906976744" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.3333333333333" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.8294573643411" style="1"/>
+    <col min="3" max="3" width="11.59375"/>
+    <col min="5" max="5" width="12.7109375"/>
+    <col min="6" max="6" width="14.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.3359375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.3359375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.8359375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="40.5" customHeight="1" spans="1:10">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:10">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="20">
         <v>5191</v>
       </c>
-      <c r="C2" s="35">
+      <c r="C2" s="46">
         <v>6571276.82</v>
       </c>
       <c r="D2" s="1">
         <v>1946</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2" s="47">
         <v>10539098.29</v>
       </c>
       <c r="F2" s="1">
@@ -1541,19 +1647,19 @@
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:10">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="36">
+      <c r="B3" s="1">
         <v>4684</v>
       </c>
-      <c r="C3" s="37">
+      <c r="C3" s="47">
         <v>8243621.3</v>
       </c>
-      <c r="D3" s="36">
+      <c r="D3" s="1">
         <v>1917</v>
       </c>
-      <c r="E3" s="37">
+      <c r="E3" s="47">
         <v>11528192.33</v>
       </c>
       <c r="F3" s="1">
@@ -1568,9 +1674,174 @@
       <c r="I3" s="1">
         <v>3925227.65</v>
       </c>
-      <c r="J3" s="38">
+      <c r="J3" s="48">
         <f>(C3-C2)/C2</f>
         <v>0.254493080387382</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:10">
+      <c r="A4" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1">
+        <v>4209</v>
+      </c>
+      <c r="C4" s="47">
+        <v>6299630.46</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1865</v>
+      </c>
+      <c r="E4" s="47">
+        <v>11679168.68</v>
+      </c>
+      <c r="F4" s="1">
+        <v>99</v>
+      </c>
+      <c r="G4" s="1">
+        <v>421603.45</v>
+      </c>
+      <c r="H4" s="1">
+        <v>302</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3451864.23</v>
+      </c>
+      <c r="J4" s="48">
+        <f>(C4-C3)/C3</f>
+        <v>-0.235817581770769</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:10">
+      <c r="A5" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3691</v>
+      </c>
+      <c r="C5" s="47">
+        <v>4858299.45</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1645</v>
+      </c>
+      <c r="E5" s="47">
+        <v>10458449.14</v>
+      </c>
+      <c r="F5" s="1">
+        <v>95</v>
+      </c>
+      <c r="G5" s="1">
+        <v>385676.99</v>
+      </c>
+      <c r="H5" s="1">
+        <v>278</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3212199.99</v>
+      </c>
+      <c r="J5" s="48">
+        <f>(C5-C4)/C4</f>
+        <v>-0.228796120526727</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:10">
+      <c r="A6" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1">
+        <v>5123</v>
+      </c>
+      <c r="C6" s="47">
+        <v>6522812.78</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2054</v>
+      </c>
+      <c r="E6" s="47">
+        <v>11997970.5</v>
+      </c>
+      <c r="F6" s="1">
+        <v>91</v>
+      </c>
+      <c r="G6" s="1">
+        <v>377824.39</v>
+      </c>
+      <c r="H6" s="1">
+        <v>252</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3011737.21</v>
+      </c>
+      <c r="J6" s="48">
+        <f>(C6-C5)/C5</f>
+        <v>0.34261233732721</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" spans="1:10">
+      <c r="A7" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="1">
+        <v>5180</v>
+      </c>
+      <c r="C7" s="47">
+        <v>7345266.86</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2449</v>
+      </c>
+      <c r="E7" s="47">
+        <v>12930932.43</v>
+      </c>
+      <c r="F7" s="1">
+        <v>88</v>
+      </c>
+      <c r="G7" s="1">
+        <v>355784.71</v>
+      </c>
+      <c r="H7" s="1">
+        <v>233</v>
+      </c>
+      <c r="I7" s="1">
+        <v>2743976.67</v>
+      </c>
+      <c r="J7" s="48">
+        <f>(C7-C6)/C6</f>
+        <v>0.126088868060383</v>
+      </c>
+    </row>
+    <row r="8" customHeight="1" spans="1:10">
+      <c r="A8" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1">
+        <v>6524</v>
+      </c>
+      <c r="C8" s="47">
+        <v>8537316.3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>2460</v>
+      </c>
+      <c r="E8" s="47">
+        <v>13335319.79</v>
+      </c>
+      <c r="F8" s="1">
+        <v>87</v>
+      </c>
+      <c r="G8" s="1">
+        <v>355524.71</v>
+      </c>
+      <c r="H8" s="1">
+        <v>218</v>
+      </c>
+      <c r="I8" s="1">
+        <v>2588635.57</v>
+      </c>
+      <c r="J8" s="48">
+        <f>(C8-C7)/C7</f>
+        <v>0.162288105077778</v>
       </c>
     </row>
   </sheetData>
@@ -1584,157 +1855,346 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="6.82945736434108" style="1" customWidth="1"/>
-    <col min="2" max="6" width="18" style="25" customWidth="1"/>
+    <col min="1" max="1" width="6.8359375" style="1" customWidth="1"/>
+    <col min="2" max="6" width="18" style="23" customWidth="1"/>
     <col min="7" max="7" width="18" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.16279069767442" style="25" customWidth="1"/>
+    <col min="8" max="8" width="9.1640625" style="23" customWidth="1"/>
     <col min="9" max="9" width="19" style="1" customWidth="1"/>
     <col min="10" max="11" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:11">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="26" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="27" t="s">
+      <c r="B1" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" customHeight="1" spans="1:11">
+      <c r="A2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="39">
+        <v>1039</v>
+      </c>
+      <c r="C2" s="39">
+        <v>2486</v>
+      </c>
+      <c r="D2" s="40">
+        <v>1169</v>
+      </c>
+      <c r="E2" s="40">
+        <v>521</v>
+      </c>
+      <c r="F2" s="41">
+        <v>0.446</v>
+      </c>
+      <c r="G2" s="10">
+        <v>4141198.82</v>
+      </c>
+      <c r="H2" s="19">
         <v>15</v>
       </c>
-      <c r="F1" s="27" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:11">
-      <c r="A2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="29">
-        <v>1039</v>
-      </c>
-      <c r="C2" s="29">
-        <v>2486</v>
-      </c>
-      <c r="D2" s="30">
+      <c r="I2" s="10">
+        <v>276079.92</v>
+      </c>
+      <c r="J2" s="10">
+        <v>165.7</v>
+      </c>
+      <c r="K2" s="42"/>
+    </row>
+    <row r="3" customHeight="1" spans="1:11">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="39">
         <v>1169</v>
       </c>
-      <c r="E2" s="30">
-        <v>521</v>
-      </c>
-      <c r="F2" s="31">
-        <v>0.446</v>
-      </c>
-      <c r="G2" s="7">
-        <v>4141198.82</v>
-      </c>
-      <c r="H2" s="32">
+      <c r="C3" s="39">
+        <v>3698</v>
+      </c>
+      <c r="D3" s="40">
+        <v>1138</v>
+      </c>
+      <c r="E3" s="40">
+        <v>515</v>
+      </c>
+      <c r="F3" s="41">
+        <v>0.453</v>
+      </c>
+      <c r="G3" s="10">
+        <v>5760008.07</v>
+      </c>
+      <c r="H3" s="19">
         <v>15</v>
       </c>
-      <c r="I2" s="7">
-        <v>276079.92</v>
-      </c>
-      <c r="J2" s="7">
-        <v>165.7</v>
-      </c>
-      <c r="K2" s="24"/>
-    </row>
-    <row r="3" customHeight="1" spans="1:11">
-      <c r="A3" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="29">
-        <v>1169</v>
-      </c>
-      <c r="C3" s="29">
-        <v>3698</v>
-      </c>
-      <c r="D3" s="30">
-        <v>1138</v>
-      </c>
-      <c r="E3" s="30">
-        <v>515</v>
-      </c>
-      <c r="F3" s="31">
-        <v>0.453</v>
-      </c>
-      <c r="G3" s="7">
-        <v>5760008.07</v>
-      </c>
-      <c r="H3" s="32">
+      <c r="I3" s="10">
+        <v>384000.54</v>
+      </c>
+      <c r="J3" s="10">
+        <v>246.5</v>
+      </c>
+      <c r="K3" s="42">
+        <v>0.391</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:11">
+      <c r="A4" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="39">
+        <v>845</v>
+      </c>
+      <c r="C4" s="39">
+        <v>2042</v>
+      </c>
+      <c r="D4" s="40">
+        <v>893</v>
+      </c>
+      <c r="E4" s="40">
+        <v>448</v>
+      </c>
+      <c r="F4" s="41">
+        <f t="shared" ref="F4:F8" si="0">E4/D4</f>
+        <v>0.501679731243001</v>
+      </c>
+      <c r="G4" s="10">
+        <v>4556368.56</v>
+      </c>
+      <c r="H4" s="19">
         <v>15</v>
       </c>
-      <c r="I3" s="7">
-        <v>384000.54</v>
-      </c>
-      <c r="J3" s="7">
-        <v>246.5</v>
-      </c>
-      <c r="K3" s="24">
-        <v>0.391</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:11">
-      <c r="A4" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="29">
-        <v>845</v>
-      </c>
-      <c r="C4" s="29">
-        <v>2042</v>
-      </c>
-      <c r="D4" s="30">
-        <v>893</v>
-      </c>
-      <c r="E4" s="30">
-        <v>448</v>
-      </c>
-      <c r="F4" s="31">
-        <f>E4/D4</f>
-        <v>0.501679731243001</v>
-      </c>
-      <c r="G4" s="7">
-        <v>4556368.56</v>
-      </c>
-      <c r="H4" s="32">
-        <v>15</v>
-      </c>
-      <c r="I4" s="7">
-        <f>G4/H4</f>
+      <c r="I4" s="10">
+        <f t="shared" ref="I4:I8" si="1">G4/H4</f>
         <v>303757.904</v>
       </c>
-      <c r="J4" s="7">
-        <f>C4/H4</f>
+      <c r="J4" s="10">
+        <f t="shared" ref="J4:J8" si="2">C4/H4</f>
         <v>136.133333333333</v>
       </c>
-      <c r="K4" s="24">
+      <c r="K4" s="42">
         <f>(G4-G3)/G3</f>
         <v>-0.208964899939802</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:11">
+      <c r="A5" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="39">
+        <v>883</v>
+      </c>
+      <c r="C5" s="39">
+        <v>2068</v>
+      </c>
+      <c r="D5" s="40">
+        <v>1016</v>
+      </c>
+      <c r="E5" s="40">
+        <v>472</v>
+      </c>
+      <c r="F5" s="41">
+        <f t="shared" si="0"/>
+        <v>0.464566929133858</v>
+      </c>
+      <c r="G5" s="10">
+        <v>5067066.46</v>
+      </c>
+      <c r="H5" s="19">
+        <v>15</v>
+      </c>
+      <c r="I5" s="10">
+        <f t="shared" si="1"/>
+        <v>337804.430666667</v>
+      </c>
+      <c r="J5" s="10">
+        <f t="shared" si="2"/>
+        <v>137.866666666667</v>
+      </c>
+      <c r="K5" s="42">
+        <f>(G5-G4)/G4</f>
+        <v>0.112084413996571</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:11">
+      <c r="A6" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="39">
+        <v>909</v>
+      </c>
+      <c r="C6" s="39">
+        <v>1887</v>
+      </c>
+      <c r="D6" s="40">
+        <v>1070</v>
+      </c>
+      <c r="E6" s="40">
+        <v>500</v>
+      </c>
+      <c r="F6" s="41">
+        <v>0.4673</v>
+      </c>
+      <c r="G6" s="10">
+        <v>3856893.47</v>
+      </c>
+      <c r="H6" s="19">
+        <v>15</v>
+      </c>
+      <c r="I6" s="10">
+        <v>257126.2</v>
+      </c>
+      <c r="J6" s="10">
+        <v>125.8</v>
+      </c>
+      <c r="K6" s="42">
+        <f>(G6-G5)/G5</f>
+        <v>-0.238831086892829</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" spans="1:11">
+      <c r="A7" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="39">
+        <v>864</v>
+      </c>
+      <c r="C7" s="39">
+        <v>2534</v>
+      </c>
+      <c r="D7" s="40">
+        <v>803</v>
+      </c>
+      <c r="E7" s="40">
+        <v>354</v>
+      </c>
+      <c r="F7" s="41">
+        <v>0.440846824408468</v>
+      </c>
+      <c r="G7" s="10">
+        <v>3869198.47</v>
+      </c>
+      <c r="H7" s="19">
+        <v>15</v>
+      </c>
+      <c r="I7" s="10">
+        <v>257946.564666667</v>
+      </c>
+      <c r="J7" s="10">
+        <v>168.933333333333</v>
+      </c>
+      <c r="K7" s="42">
+        <f>(G7-G6)/G6</f>
+        <v>0.00319039146289928</v>
+      </c>
+    </row>
+    <row r="8" customHeight="1" spans="1:11">
+      <c r="A8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="39">
+        <v>1135</v>
+      </c>
+      <c r="C8" s="39">
+        <v>2403</v>
+      </c>
+      <c r="D8" s="40">
+        <v>1329</v>
+      </c>
+      <c r="E8" s="40">
+        <v>688</v>
+      </c>
+      <c r="F8" s="41">
+        <f t="shared" si="0"/>
+        <v>0.517682468021068</v>
+      </c>
+      <c r="G8" s="10">
+        <v>5454644.26</v>
+      </c>
+      <c r="H8" s="19">
+        <v>15</v>
+      </c>
+      <c r="I8" s="10">
+        <f t="shared" si="1"/>
+        <v>363642.950666667</v>
+      </c>
+      <c r="J8" s="10">
+        <f t="shared" si="2"/>
+        <v>160.2</v>
+      </c>
+      <c r="K8" s="42">
+        <f>(G8-G7)/G7</f>
+        <v>0.409760781798303</v>
+      </c>
+    </row>
+    <row r="9" customHeight="1" spans="1:11">
+      <c r="A9" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="39">
+        <v>1124</v>
+      </c>
+      <c r="C9" s="39">
+        <v>2712</v>
+      </c>
+      <c r="D9" s="40">
+        <v>1298</v>
+      </c>
+      <c r="E9" s="40">
+        <v>582</v>
+      </c>
+      <c r="F9" s="41">
+        <f>E9/D9</f>
+        <v>0.448382126348228</v>
+      </c>
+      <c r="G9" s="10">
+        <v>5147364.08</v>
+      </c>
+      <c r="H9" s="19">
+        <v>15</v>
+      </c>
+      <c r="I9" s="10">
+        <f>G9/H9</f>
+        <v>343157.605333333</v>
+      </c>
+      <c r="J9" s="10">
+        <f>C9/H9</f>
+        <v>180.8</v>
+      </c>
+      <c r="K9" s="42">
+        <f>(G9-G8)/G8</f>
+        <v>-0.0563336792196233</v>
       </c>
     </row>
   </sheetData>
@@ -1749,77 +2209,88 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="4"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="7" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="5" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:5">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>27</v>
+      <c r="B1" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:5">
-      <c r="A2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="5">
-        <v>2264</v>
-      </c>
-      <c r="C2" s="5">
-        <v>48</v>
-      </c>
-      <c r="D2" s="24">
-        <v>0.0212</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>28</v>
+      <c r="A2" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>3183</v>
+      </c>
+      <c r="C2">
+        <v>71</v>
+      </c>
+      <c r="D2" s="35">
+        <f>C2/B2</f>
+        <v>0.022306000628338</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:5">
-      <c r="A3" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="5">
-        <v>2248</v>
-      </c>
-      <c r="C3" s="5">
-        <v>69</v>
-      </c>
-      <c r="D3" s="24">
-        <v>0.0307</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="A3"/>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
     </row>
     <row r="4" customHeight="1" spans="1:5">
-      <c r="A4" s="40" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="5">
-        <v>2248</v>
-      </c>
-      <c r="C4" s="1">
-        <v>46</v>
-      </c>
-      <c r="D4" s="24">
-        <f>C4/B4</f>
-        <v>0.0204626334519573</v>
-      </c>
+      <c r="A4"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+    </row>
+    <row r="5" customHeight="1" spans="1:5">
+      <c r="A5"/>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+    </row>
+    <row r="6" customHeight="1" spans="1:5">
+      <c r="A6"/>
+      <c r="B6"/>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6"/>
+    </row>
+    <row r="7" customHeight="1" spans="1:5">
+      <c r="A7"/>
+      <c r="B7"/>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+    </row>
+    <row r="8" customHeight="1" spans="1:5">
+      <c r="A8"/>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1832,67 +2303,142 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="4" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:4">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>32</v>
+      <c r="B1" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:4">
-      <c r="A2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="7">
+      <c r="A2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="10">
         <v>4971.97</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="10">
         <v>56502.88</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="10">
         <v>61474.85</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:4">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="10">
         <v>5210.54</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="10">
         <v>25998.03</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="10">
         <v>31208.57</v>
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:4">
-      <c r="A4" s="40" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="7">
+      <c r="A4" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="10">
         <v>17901.513</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="10">
         <v>5144.33</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="10">
         <f>B4+C4</f>
         <v>23045.843</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:4">
+      <c r="A5" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="10">
+        <v>8965.11</v>
+      </c>
+      <c r="C5" s="10">
+        <v>41747.28</v>
+      </c>
+      <c r="D5" s="10">
+        <f>B5+C5</f>
+        <v>50712.39</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:4">
+      <c r="A6" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="10">
+        <v>9220.52</v>
+      </c>
+      <c r="C6" s="10">
+        <v>9011.29</v>
+      </c>
+      <c r="D6" s="10">
+        <f>B6+C6</f>
+        <v>18231.81</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" spans="1:4">
+      <c r="A7" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="10">
+        <v>4373.05</v>
+      </c>
+      <c r="C7" s="10">
+        <v>56280.08</v>
+      </c>
+      <c r="D7" s="10">
+        <f>B7+C7</f>
+        <v>60653.13</v>
+      </c>
+    </row>
+    <row r="8" customHeight="1" spans="1:4">
+      <c r="A8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1">
+        <v>7087.52</v>
+      </c>
+      <c r="C8" s="1">
+        <v>103017.42</v>
+      </c>
+      <c r="D8" s="10">
+        <f>B8+C8</f>
+        <v>110104.94</v>
+      </c>
+    </row>
+    <row r="9" customHeight="1" spans="1:4">
+      <c r="A9" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1">
+        <v>10527.14</v>
+      </c>
+      <c r="C9" s="1">
+        <v>5511</v>
+      </c>
+      <c r="D9" s="10">
+        <f>B9+C9</f>
+        <v>16038.14</v>
       </c>
     </row>
   </sheetData>
@@ -1906,181 +2452,248 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="2"/>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="18" style="1" customWidth="1"/>
-    <col min="2" max="5" width="14.1627906976744" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.3333333333333" style="1" customWidth="1"/>
-    <col min="7" max="9" width="14.1627906976744" style="1" customWidth="1"/>
-    <col min="10" max="13" width="12.8294573643411" style="1"/>
+    <col min="2" max="5" width="14.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.3359375" style="25" customWidth="1"/>
+    <col min="7" max="9" width="14.1640625" style="25" customWidth="1"/>
+    <col min="10" max="13" width="12.8359375" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" customHeight="1" spans="1:17">
-      <c r="A1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="15" t="s">
+    <row r="1" s="4" customFormat="1" customHeight="1" spans="1:17">
+      <c r="A1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="B1" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="C1" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="D1" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="E1" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="F1" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="G1" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="H1" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="I1" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="J1" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="O1" s="15" t="s">
+      <c r="K1" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="P1" s="15" t="s">
+      <c r="L1" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="Q1" s="15" t="s">
+      <c r="M1" s="28" t="s">
         <v>49</v>
       </c>
+      <c r="N1" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="O1" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="P1" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q1" s="26" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="2" customHeight="1" spans="1:17">
-      <c r="A2" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="19">
+      <c r="A2" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="30">
         <v>8446</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="30">
         <v>1301</v>
       </c>
-      <c r="D2" s="19">
+      <c r="D2" s="30">
         <v>1040</v>
       </c>
-      <c r="E2" s="19">
+      <c r="E2" s="30">
         <v>1202</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="31">
         <v>1814.43594600995</v>
       </c>
-      <c r="G2" s="20">
+      <c r="G2" s="31">
         <v>1091.67947732513</v>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="31">
         <v>558.466346153846</v>
       </c>
-      <c r="I2" s="20">
+      <c r="I2" s="31">
         <v>519.371048252912</v>
       </c>
-      <c r="J2" s="21">
+      <c r="J2" s="32">
         <v>543.79694529955</v>
       </c>
-      <c r="K2" s="21">
+      <c r="K2" s="32">
         <v>289.948501152959</v>
       </c>
-      <c r="L2" s="21">
+      <c r="L2" s="32">
         <v>197.801923076923</v>
       </c>
-      <c r="M2" s="21">
+      <c r="M2" s="32">
         <v>184.280366056572</v>
       </c>
-      <c r="N2" s="19">
+      <c r="N2" s="30">
         <v>225323</v>
       </c>
-      <c r="O2" s="19">
+      <c r="O2" s="30">
         <v>33193</v>
       </c>
-      <c r="P2" s="19">
+      <c r="P2" s="30">
         <v>24736</v>
       </c>
-      <c r="Q2" s="19">
+      <c r="Q2" s="30">
         <v>22844</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:17">
-      <c r="A3" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="19">
+      <c r="A3" s="52" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="30">
         <v>8446</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="30">
         <v>1100</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="30">
         <v>1040</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="30">
         <v>1202</v>
       </c>
-      <c r="F3" s="22">
+      <c r="F3" s="33">
         <f>18279769/B3</f>
         <v>2164.31079801089</v>
       </c>
-      <c r="G3" s="22">
+      <c r="G3" s="33">
         <f>2542454/C3</f>
         <v>2311.32181818182</v>
       </c>
-      <c r="H3" s="22">
+      <c r="H3" s="33">
         <f>727465/D3</f>
         <v>699.485576923077</v>
       </c>
-      <c r="I3" s="22">
+      <c r="I3" s="33">
         <f>955153/E3</f>
         <v>794.636439267887</v>
       </c>
-      <c r="J3" s="23">
+      <c r="J3" s="34">
         <f>5257975/B3</f>
         <v>622.540255742363</v>
       </c>
-      <c r="K3" s="23">
+      <c r="K3" s="34">
         <f>629021/C3</f>
         <v>571.837272727273</v>
       </c>
-      <c r="L3" s="23">
+      <c r="L3" s="34">
         <f>251054/D3</f>
         <v>241.398076923077</v>
       </c>
-      <c r="M3" s="23">
+      <c r="M3" s="34">
         <f>275215/E3</f>
         <v>228.964226289517</v>
       </c>
-      <c r="N3" s="19">
+      <c r="N3" s="30">
         <v>225323</v>
       </c>
-      <c r="O3" s="19">
-        <v>33193</v>
-      </c>
-      <c r="P3" s="19">
+      <c r="O3" s="30">
+        <v>20000</v>
+      </c>
+      <c r="P3" s="30">
         <v>24736</v>
       </c>
-      <c r="Q3" s="19">
+      <c r="Q3" s="30">
         <v>22844</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:17">
+      <c r="A4" s="52" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="30">
+        <v>8446</v>
+      </c>
+      <c r="C4" s="30">
+        <v>1100</v>
+      </c>
+      <c r="D4" s="30">
+        <v>1040</v>
+      </c>
+      <c r="E4" s="30">
+        <v>1202</v>
+      </c>
+      <c r="F4" s="33">
+        <f>16047133/B3</f>
+        <v>1899.96838740232</v>
+      </c>
+      <c r="G4" s="33">
+        <f>2214298/C3</f>
+        <v>2012.99818181818</v>
+      </c>
+      <c r="H4" s="33">
+        <f>443140/D3</f>
+        <v>426.096153846154</v>
+      </c>
+      <c r="I4" s="33">
+        <f>718500/E3</f>
+        <v>597.753743760399</v>
+      </c>
+      <c r="J4" s="34">
+        <f>4565965/B3</f>
+        <v>540.606796116505</v>
+      </c>
+      <c r="K4" s="34">
+        <f>550000/C3</f>
+        <v>500</v>
+      </c>
+      <c r="L4" s="34">
+        <f>156175/D3</f>
+        <v>150.168269230769</v>
+      </c>
+      <c r="M4" s="34">
+        <f>202780/E3</f>
+        <v>168.702163061564</v>
+      </c>
+      <c r="N4" s="30">
+        <v>225323</v>
+      </c>
+      <c r="O4" s="30">
+        <v>20000</v>
+      </c>
+      <c r="P4" s="30">
+        <v>24736</v>
+      </c>
+      <c r="Q4" s="30">
+        <v>22844</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:17">
+      <c r="N6">
+        <f>29.3*0.12</f>
+        <v>3.516</v>
       </c>
     </row>
   </sheetData>
@@ -2094,57 +2707,115 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="2"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.8294573643411" style="1" customWidth="1"/>
-    <col min="3" max="3" width="39.6666666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.8359375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="65.9765625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>53</v>
+      <c r="B1" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:3">
-      <c r="A2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>55</v>
+      <c r="A2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" ht="229.5" customHeight="1" spans="1:3">
-      <c r="A4" s="13" t="s">
+      <c r="B3" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" ht="168" customHeight="1" spans="1:3">
+      <c r="A4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="B4" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" ht="146" customHeight="1" spans="1:3">
+      <c r="A5" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" ht="114" customHeight="1" spans="1:3">
+      <c r="A6" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" customHeight="1" spans="1:3">
+      <c r="A7" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" ht="43" customHeight="1" spans="1:3">
+      <c r="A8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1" spans="1:3">
+      <c r="A9" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1" spans="1:3">
+      <c r="C11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2157,305 +2828,459 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1"/>
+  <dimension ref="A1:Q8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="7"/>
   <cols>
-    <col min="1" max="1" width="21.3333333333333" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.8294573643411" style="3" customWidth="1"/>
-    <col min="3" max="3" width="15.6666666666667" style="3" customWidth="1"/>
-    <col min="4" max="6" width="13.8294573643411" style="3" customWidth="1"/>
-    <col min="7" max="7" width="17.1627906976744" style="1" customWidth="1"/>
-    <col min="8" max="11" width="12.4961240310078" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.328125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="13.828125" style="4" customWidth="1"/>
+    <col min="8" max="11" width="12.5" style="1" customWidth="1"/>
+    <col min="16" max="16" width="13.828125"/>
+    <col min="17" max="17" width="13.828125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" ht="27" customHeight="1" spans="1:11">
-      <c r="A1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:11">
-      <c r="A2" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" s="6">
+    <row r="1" s="4" customFormat="1" ht="27.75" customHeight="1" spans="1:17">
+      <c r="A1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" customHeight="1" spans="1:17">
+      <c r="A2" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="8">
         <v>12960913.76</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="8">
         <v>59780928.78</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="9">
         <v>4.61</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="9">
         <v>79.1</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="8">
         <v>14129745.66</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="8">
         <v>57251892.44</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="10">
         <v>4.05</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="10">
         <v>90.1</v>
       </c>
-      <c r="J2" s="8">
+      <c r="J2" s="11">
         <v>0.09</v>
       </c>
-      <c r="K2" s="7">
+      <c r="K2" s="10">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:11">
-      <c r="A3" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" s="6">
+      <c r="L2" s="8">
+        <v>16098978.5200001</v>
+      </c>
+      <c r="M2" s="8">
+        <v>72676746.52</v>
+      </c>
+      <c r="N2" s="12">
+        <v>4.51437005333675</v>
+      </c>
+      <c r="O2" s="12">
+        <v>80.8529198288063</v>
+      </c>
+      <c r="P2" s="13">
+        <f>(L2-F2)/F2</f>
+        <v>0.139367891495373</v>
+      </c>
+      <c r="Q2" s="14">
+        <f>O2-I2</f>
+        <v>-9.2470801711937</v>
+      </c>
+    </row>
+    <row r="3" customHeight="1" spans="1:17">
+      <c r="A3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="15">
         <v>32900585.42</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="15">
         <v>134744245.49</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="9">
         <v>4.1</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="9">
         <v>89.1</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="15">
         <v>34198877.49</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="15">
         <v>131835427.48</v>
       </c>
-      <c r="H3" s="7">
+      <c r="H3" s="10">
         <v>3.85</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="10">
         <v>94.7</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="11">
         <v>0.039</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="10">
         <v>5.6</v>
       </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:11">
-      <c r="A4" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="L3" s="8">
+        <v>35864929.5309738</v>
+      </c>
+      <c r="M3" s="15">
+        <v>137069373.96</v>
+      </c>
+      <c r="N3" s="12">
+        <v>3.82182192332551</v>
+      </c>
+      <c r="O3" s="12">
+        <v>95.5041881392528</v>
+      </c>
+      <c r="P3" s="13">
+        <f t="shared" ref="P3:P8" si="0">(L3-F3)/F3</f>
+        <v>0.0487165709301705</v>
+      </c>
+      <c r="Q3" s="14">
+        <f t="shared" ref="Q3:Q8" si="1">O3-I3</f>
+        <v>0.804188139252801</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:17">
+      <c r="A4" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="15">
         <v>1979750.45</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="15">
         <v>14321547.68</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="9">
         <v>7.23</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="9">
         <v>50.5</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="15">
         <v>1851979.97</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="15">
         <v>13356804.36</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="10">
         <v>7.21</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="10">
         <v>50.6</v>
       </c>
-      <c r="J4" s="8">
+      <c r="J4" s="11">
         <v>-0.065</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="10">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:11">
-      <c r="A5" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="L4" s="8">
+        <v>1851979.96999999</v>
+      </c>
+      <c r="M4" s="15">
+        <v>12940895.152</v>
+      </c>
+      <c r="N4" s="12">
+        <v>6.98759995336238</v>
+      </c>
+      <c r="O4" s="12">
+        <v>52.2353887509494</v>
+      </c>
+      <c r="P4" s="13">
+        <f t="shared" si="0"/>
+        <v>-5.40595354123425e-15</v>
+      </c>
+      <c r="Q4" s="14">
+        <f t="shared" si="1"/>
+        <v>1.6353887509494</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:17">
+      <c r="A5" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="15">
         <v>3506939.44</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="15">
         <v>31251759.68</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="4">
         <v>8.91</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="9">
         <v>41</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="15">
         <v>3502534.97</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="15">
         <v>32057459.56</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="10">
         <v>9.15</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="10">
         <v>39.9</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="11">
         <v>-0.001</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="10">
         <v>-1.1</v>
       </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:11">
-      <c r="A6" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="6">
+      <c r="L5" s="8">
+        <v>3335920.32743364</v>
+      </c>
+      <c r="M5" s="15">
+        <v>33775261.768</v>
+      </c>
+      <c r="N5" s="12">
+        <v>10.1247207525438</v>
+      </c>
+      <c r="O5" s="12">
+        <v>36.0503769852908</v>
+      </c>
+      <c r="P5" s="13">
+        <f t="shared" si="0"/>
+        <v>-0.047569729922314</v>
+      </c>
+      <c r="Q5" s="14">
+        <f t="shared" si="1"/>
+        <v>-3.8496230147092</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:17">
+      <c r="A6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="15">
         <v>1367089.88</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="15">
         <v>14437535.33</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="4">
         <v>10.56</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="9">
         <v>34.6</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="15">
         <v>1345513.08</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="15">
         <v>12785473.64</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="10">
         <v>9.5</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="10">
         <v>38.4</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="11">
         <v>-0.016</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="10">
         <v>3.8</v>
       </c>
-    </row>
-    <row r="7" ht="14.25" customHeight="1" spans="1:11">
+      <c r="L6" s="8">
+        <v>1361927.36283185</v>
+      </c>
+      <c r="M6" s="15">
+        <v>11901326.796</v>
+      </c>
+      <c r="N6" s="12">
+        <v>8.73859144092209</v>
+      </c>
+      <c r="O6" s="12">
+        <v>41.7687452797868</v>
+      </c>
+      <c r="P6" s="13">
+        <f t="shared" si="0"/>
+        <v>0.0121992740730919</v>
+      </c>
+      <c r="Q6" s="14">
+        <f t="shared" si="1"/>
+        <v>3.3687452797868</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25" customHeight="1" spans="1:17">
       <c r="A7" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="6">
+        <v>91</v>
+      </c>
+      <c r="B7" s="15">
         <v>11818000</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="16">
         <v>0</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="17">
         <v>0</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="17">
         <v>0</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="15">
         <v>11747000</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="16">
         <v>0</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="17">
         <v>0</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="17">
         <v>0</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="17">
         <v>0</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="17">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" ht="14.25" customHeight="1" spans="1:11">
+      <c r="L7" s="8">
+        <v>11691690.6194693</v>
+      </c>
+      <c r="M7" s="16">
+        <v>0</v>
+      </c>
+      <c r="N7" s="12">
+        <v>0</v>
+      </c>
+      <c r="O7" s="12">
+        <v>0</v>
+      </c>
+      <c r="P7" s="13">
+        <f t="shared" si="0"/>
+        <v>-0.00470838346222015</v>
+      </c>
+      <c r="Q7" s="14">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25" customHeight="1" spans="1:17">
       <c r="A8" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="6">
+        <v>92</v>
+      </c>
+      <c r="B8" s="15">
         <f>SUM(B3:B7)</f>
         <v>51572365.19</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="15">
         <f>SUM(C3:C7)</f>
         <v>194755088.18</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="17">
         <f>C8/B8</f>
         <v>3.77634586784016</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="17">
         <v>98.6</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="15">
         <f>SUM(F3:F7)</f>
         <v>52645905.51</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="15">
         <f>SUM(G3:G7)</f>
         <v>190035165.04</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="17">
         <f>G8/F8</f>
         <v>3.60968556242048</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="17">
         <v>103</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="17">
         <v>0.019</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="17">
         <v>4.4</v>
       </c>
-    </row>
-    <row r="9" customHeight="1" spans="1:11">
-      <c r="F9" s="9"/>
+      <c r="L8" s="8">
+        <v>54106447.8107086</v>
+      </c>
+      <c r="M8" s="15">
+        <v>195686857.676</v>
+      </c>
+      <c r="N8" s="12">
+        <v>3.61670125454568</v>
+      </c>
+      <c r="O8" s="12">
+        <v>100.920693834263</v>
+      </c>
+      <c r="P8" s="13">
+        <f t="shared" si="0"/>
+        <v>0.0277427520062538</v>
+      </c>
+      <c r="Q8" s="14">
+        <f t="shared" si="1"/>
+        <v>-2.07930616573699</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2468,44 +3293,28 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="3" outlineLevelCol="1"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" customHeight="1" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="28.5038759689922" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.1627906976744" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.6666666666667" style="1" customWidth="1"/>
+    <col min="2" max="2" width="126.2734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:2">
-      <c r="A2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:2">
-      <c r="A3" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2222</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:2">
-      <c r="A4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="1">
-        <v>666</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" customFormat="1" ht="20" customHeight="1" spans="1:2">
+      <c r="A2" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>